<commit_message>
Add Testing doc, bug lifecycle, techniques
</commit_message>
<xml_diff>
--- a/Others/Testing levels comparison.xlsx
+++ b/Others/Testing levels comparison.xlsx
@@ -1,15 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
-  <fileVersion appName="xl" lastEdited="6" lowestEdited="6" rupBuild="14420"/>
-  <workbookPr defaultThemeVersion="164011"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29127"/>
+  <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Storage\Study Notes\study-notes\Others\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Projects\study-notes\Others\"/>
     </mc:Choice>
   </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7B19815D-2141-4F8A-817A-B37414F26446}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="23040" windowHeight="9072" activeTab="3"/>
+    <workbookView xWindow="-180" yWindow="-180" windowWidth="19560" windowHeight="10440" firstSheet="2" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Tools" sheetId="8" r:id="rId1"/>
@@ -3278,7 +3279,7 @@
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <fonts count="10" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
@@ -3629,6 +3630,21 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -3652,21 +3668,6 @@
     </xf>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -3702,7 +3703,13 @@
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="2" name="Picture 1"/>
+        <xdr:cNvPr id="2" name="Picture 1">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0200-000002000000}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
         <xdr:cNvPicPr>
           <a:picLocks noChangeAspect="1"/>
         </xdr:cNvPicPr>
@@ -3740,7 +3747,13 @@
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="3" name="Picture 2" descr="SDLC - V Model - Notepub"/>
+        <xdr:cNvPr id="3" name="Picture 2" descr="SDLC - V Model - Notepub">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0200-000003000000}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
         <xdr:cNvPicPr>
           <a:picLocks noChangeAspect="1" noChangeArrowheads="1"/>
         </xdr:cNvPicPr>
@@ -3795,7 +3808,13 @@
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="4" name="Picture 3" descr="Iterative and incremental development - Wikipedia"/>
+        <xdr:cNvPr id="4" name="Picture 3" descr="Iterative and incremental development - Wikipedia">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0200-000004000000}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
         <xdr:cNvPicPr>
           <a:picLocks noChangeAspect="1" noChangeArrowheads="1"/>
         </xdr:cNvPicPr>
@@ -3850,7 +3869,13 @@
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="5" name="Picture 4" descr="The Agile Software Development Life Cycle | Wrike Agile Guide"/>
+        <xdr:cNvPr id="5" name="Picture 4" descr="The Agile Software Development Life Cycle | Wrike Agile Guide">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0200-000005000000}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
         <xdr:cNvPicPr>
           <a:picLocks noChangeAspect="1" noChangeArrowheads="1"/>
         </xdr:cNvPicPr>
@@ -3903,7 +3928,13 @@
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="6" name="Picture 5" descr="DevOps: the pillars to accelerate the SDLC | Mia-Platform"/>
+        <xdr:cNvPr id="6" name="Picture 5" descr="DevOps: the pillars to accelerate the SDLC | Mia-Platform">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0200-000006000000}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
         <xdr:cNvPicPr>
           <a:picLocks noChangeAspect="1" noChangeArrowheads="1"/>
         </xdr:cNvPicPr>
@@ -4217,19 +4248,19 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:F14"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="23" customWidth="1"/>
-    <col min="2" max="2" width="27.6640625" customWidth="1"/>
-    <col min="3" max="3" width="25.44140625" customWidth="1"/>
-    <col min="4" max="4" width="27.88671875" customWidth="1"/>
+    <col min="2" max="2" width="27.6328125" customWidth="1"/>
+    <col min="3" max="3" width="25.453125" customWidth="1"/>
+    <col min="4" max="4" width="27.90625" customWidth="1"/>
     <col min="5" max="5" width="24" style="5" customWidth="1"/>
     <col min="6" max="6" width="26" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A1" s="55" t="s">
         <v>288</v>
       </c>
@@ -4245,18 +4276,18 @@
       <c r="E1" s="55" t="s">
         <v>292</v>
       </c>
-      <c r="F1" s="65" t="s">
+      <c r="F1" s="57" t="s">
         <v>333</v>
       </c>
     </row>
-    <row r="2" spans="1:6" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:6" ht="29" x14ac:dyDescent="0.35">
       <c r="A2" s="25" t="s">
         <v>293</v>
       </c>
       <c r="B2" s="26" t="s">
         <v>294</v>
       </c>
-      <c r="C2" s="64" t="s">
+      <c r="C2" s="56" t="s">
         <v>295</v>
       </c>
       <c r="D2" s="26" t="s">
@@ -4266,7 +4297,7 @@
         <v>297</v>
       </c>
     </row>
-    <row r="3" spans="1:6" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:6" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A3" s="25" t="s">
         <v>298</v>
       </c>
@@ -4282,11 +4313,11 @@
       <c r="E3" s="26" t="s">
         <v>301</v>
       </c>
-      <c r="F3" s="66" t="s">
+      <c r="F3" s="58" t="s">
         <v>334</v>
       </c>
     </row>
-    <row r="4" spans="1:6" ht="57.6" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:6" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A4" s="25" t="s">
         <v>302</v>
       </c>
@@ -4302,11 +4333,11 @@
       <c r="E4" s="51" t="s">
         <v>306</v>
       </c>
-      <c r="F4" s="66" t="s">
+      <c r="F4" s="58" t="s">
         <v>335</v>
       </c>
     </row>
-    <row r="5" spans="1:6" ht="43.2" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:6" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A5" s="25" t="s">
         <v>307</v>
       </c>
@@ -4322,11 +4353,11 @@
       <c r="E5" s="26" t="s">
         <v>311</v>
       </c>
-      <c r="F5" s="66" t="s">
+      <c r="F5" s="58" t="s">
         <v>336</v>
       </c>
     </row>
-    <row r="6" spans="1:6" ht="100.8" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:6" ht="72.5" x14ac:dyDescent="0.35">
       <c r="A6" s="25" t="s">
         <v>337</v>
       </c>
@@ -4334,11 +4365,11 @@
       <c r="C6" s="26"/>
       <c r="D6" s="26"/>
       <c r="E6" s="26"/>
-      <c r="F6" s="68" t="s">
+      <c r="F6" s="59" t="s">
         <v>338</v>
       </c>
     </row>
-    <row r="7" spans="1:6" ht="43.2" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:6" ht="29" x14ac:dyDescent="0.35">
       <c r="A7" s="25" t="s">
         <v>312</v>
       </c>
@@ -4355,7 +4386,7 @@
         <v>316</v>
       </c>
     </row>
-    <row r="8" spans="1:6" ht="43.2" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:6" ht="29" x14ac:dyDescent="0.35">
       <c r="A8" s="25" t="s">
         <v>317</v>
       </c>
@@ -4366,7 +4397,7 @@
         <v>318</v>
       </c>
     </row>
-    <row r="9" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A9" s="25" t="s">
         <v>319</v>
       </c>
@@ -4381,7 +4412,7 @@
         <v>322</v>
       </c>
     </row>
-    <row r="10" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A10" s="25" t="s">
         <v>323</v>
       </c>
@@ -4392,7 +4423,7 @@
         <v>324</v>
       </c>
     </row>
-    <row r="11" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A11" s="25" t="s">
         <v>325</v>
       </c>
@@ -4407,7 +4438,7 @@
         <v>326</v>
       </c>
     </row>
-    <row r="12" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:6" ht="29" x14ac:dyDescent="0.35">
       <c r="A12" s="25" t="s">
         <v>327</v>
       </c>
@@ -4422,13 +4453,13 @@
       </c>
       <c r="E12" s="51"/>
     </row>
-    <row r="14" spans="1:6" ht="78" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A14" s="67" t="s">
+    <row r="14" spans="1:6" ht="78" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A14" s="60" t="s">
         <v>331</v>
       </c>
-      <c r="B14" s="67"/>
-      <c r="C14" s="67"/>
-      <c r="D14" s="67"/>
+      <c r="B14" s="60"/>
+      <c r="C14" s="60"/>
+      <c r="D14" s="60"/>
       <c r="E14" s="53"/>
     </row>
   </sheetData>
@@ -4441,21 +4472,21 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1:H7"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="15.5546875" style="2" customWidth="1"/>
-    <col min="2" max="2" width="21.21875" style="3" customWidth="1"/>
-    <col min="3" max="3" width="36.88671875" style="3" customWidth="1"/>
-    <col min="4" max="4" width="34.77734375" style="3" customWidth="1"/>
-    <col min="5" max="5" width="13.44140625" style="2" customWidth="1"/>
-    <col min="6" max="6" width="21.6640625" style="2" customWidth="1"/>
-    <col min="7" max="7" width="19.44140625" style="2" customWidth="1"/>
-    <col min="8" max="8" width="8.88671875" style="2"/>
+    <col min="1" max="1" width="15.54296875" style="2" customWidth="1"/>
+    <col min="2" max="2" width="21.1796875" style="3" customWidth="1"/>
+    <col min="3" max="3" width="36.90625" style="3" customWidth="1"/>
+    <col min="4" max="4" width="34.81640625" style="3" customWidth="1"/>
+    <col min="5" max="5" width="13.453125" style="2" customWidth="1"/>
+    <col min="6" max="6" width="21.6328125" style="2" customWidth="1"/>
+    <col min="7" max="7" width="19.453125" style="2" customWidth="1"/>
+    <col min="8" max="8" width="8.90625" style="2"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" s="4" customFormat="1" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:8" s="4" customFormat="1" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A1" s="6" t="s">
         <v>0</v>
       </c>
@@ -4479,7 +4510,7 @@
       </c>
       <c r="H1" s="6"/>
     </row>
-    <row r="2" spans="1:8" ht="55.8" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:8" ht="55.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A2" s="8" t="s">
         <v>1</v>
       </c>
@@ -4498,14 +4529,14 @@
       <c r="F2" s="11" t="s">
         <v>27</v>
       </c>
-      <c r="G2" s="57" t="s">
+      <c r="G2" s="62" t="s">
         <v>33</v>
       </c>
-      <c r="H2" s="57" t="s">
+      <c r="H2" s="62" t="s">
         <v>24</v>
       </c>
     </row>
-    <row r="3" spans="1:8" ht="66.599999999999994" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:8" ht="66.650000000000006" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A3" s="8" t="s">
         <v>2</v>
       </c>
@@ -4524,11 +4555,11 @@
       <c r="F3" s="11" t="s">
         <v>28</v>
       </c>
-      <c r="G3" s="57"/>
-      <c r="H3" s="57"/>
-    </row>
-    <row r="4" spans="1:8" ht="51.6" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A4" s="56" t="s">
+      <c r="G3" s="62"/>
+      <c r="H3" s="62"/>
+    </row>
+    <row r="4" spans="1:8" ht="51.65" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A4" s="61" t="s">
         <v>3</v>
       </c>
       <c r="B4" s="9" t="s">
@@ -4540,7 +4571,7 @@
       <c r="D4" s="10" t="s">
         <v>44</v>
       </c>
-      <c r="E4" s="57" t="s">
+      <c r="E4" s="62" t="s">
         <v>9</v>
       </c>
       <c r="F4" s="11" t="s">
@@ -4549,10 +4580,10 @@
       <c r="G4" s="11" t="s">
         <v>34</v>
       </c>
-      <c r="H4" s="57"/>
-    </row>
-    <row r="5" spans="1:8" ht="51.6" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A5" s="56"/>
+      <c r="H4" s="62"/>
+    </row>
+    <row r="5" spans="1:8" ht="51.65" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A5" s="61"/>
       <c r="B5" s="9" t="s">
         <v>18</v>
       </c>
@@ -4562,18 +4593,18 @@
       <c r="D5" s="10" t="s">
         <v>45</v>
       </c>
-      <c r="E5" s="57"/>
+      <c r="E5" s="62"/>
       <c r="F5" s="11" t="s">
         <v>30</v>
       </c>
       <c r="G5" s="11" t="s">
         <v>35</v>
       </c>
-      <c r="H5" s="57" t="s">
+      <c r="H5" s="62" t="s">
         <v>25</v>
       </c>
     </row>
-    <row r="6" spans="1:8" ht="67.2" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:8" ht="67.25" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A6" s="8" t="s">
         <v>4</v>
       </c>
@@ -4595,9 +4626,9 @@
       <c r="G6" s="11" t="s">
         <v>36</v>
       </c>
-      <c r="H6" s="57"/>
-    </row>
-    <row r="7" spans="1:8" ht="82.2" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="H6" s="62"/>
+    </row>
+    <row r="7" spans="1:8" ht="82.25" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A7" s="8" t="s">
         <v>5</v>
       </c>
@@ -4619,7 +4650,7 @@
       <c r="G7" s="11" t="s">
         <v>37</v>
       </c>
-      <c r="H7" s="57"/>
+      <c r="H7" s="62"/>
     </row>
   </sheetData>
   <mergeCells count="5">
@@ -4635,19 +4666,19 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
   <dimension ref="A1:F12"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="21.6640625" customWidth="1"/>
-    <col min="2" max="2" width="30.77734375" customWidth="1"/>
-    <col min="3" max="3" width="37.109375" customWidth="1"/>
-    <col min="4" max="4" width="34.5546875" customWidth="1"/>
-    <col min="5" max="5" width="34.33203125" customWidth="1"/>
-    <col min="6" max="6" width="37.21875" customWidth="1"/>
+    <col min="1" max="1" width="21.6328125" customWidth="1"/>
+    <col min="2" max="2" width="30.81640625" customWidth="1"/>
+    <col min="3" max="3" width="37.08984375" customWidth="1"/>
+    <col min="4" max="4" width="34.54296875" customWidth="1"/>
+    <col min="5" max="5" width="34.36328125" customWidth="1"/>
+    <col min="6" max="6" width="37.1796875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A1" s="21" t="s">
         <v>162</v>
       </c>
@@ -4667,7 +4698,7 @@
         <v>167</v>
       </c>
     </row>
-    <row r="2" spans="1:6" ht="182.4" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:6" ht="182.4" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A2" s="21" t="s">
         <v>226</v>
       </c>
@@ -4679,7 +4710,7 @@
         <v>228</v>
       </c>
     </row>
-    <row r="3" spans="1:6" ht="65.400000000000006" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:6" ht="65.400000000000006" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A3" s="25" t="s">
         <v>168</v>
       </c>
@@ -4699,7 +4730,7 @@
         <v>223</v>
       </c>
     </row>
-    <row r="4" spans="1:6" ht="43.2" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:6" ht="43.25" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A4" s="25" t="s">
         <v>169</v>
       </c>
@@ -4719,7 +4750,7 @@
         <v>172</v>
       </c>
     </row>
-    <row r="5" spans="1:6" ht="45" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:6" ht="45" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A5" s="25" t="s">
         <v>173</v>
       </c>
@@ -4739,7 +4770,7 @@
         <v>178</v>
       </c>
     </row>
-    <row r="6" spans="1:6" ht="42" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:6" ht="42" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A6" s="25" t="s">
         <v>179</v>
       </c>
@@ -4759,7 +4790,7 @@
         <v>182</v>
       </c>
     </row>
-    <row r="7" spans="1:6" ht="68.400000000000006" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:6" ht="68.400000000000006" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A7" s="25" t="s">
         <v>183</v>
       </c>
@@ -4779,7 +4810,7 @@
         <v>188</v>
       </c>
     </row>
-    <row r="8" spans="1:6" ht="54.6" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:6" ht="54.65" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A8" s="25" t="s">
         <v>189</v>
       </c>
@@ -4799,7 +4830,7 @@
         <v>194</v>
       </c>
     </row>
-    <row r="9" spans="1:6" ht="42.6" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:6" ht="42.65" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A9" s="25" t="s">
         <v>195</v>
       </c>
@@ -4819,7 +4850,7 @@
         <v>200</v>
       </c>
     </row>
-    <row r="10" spans="1:6" ht="52.8" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:6" ht="52.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A10" s="25" t="s">
         <v>201</v>
       </c>
@@ -4839,7 +4870,7 @@
         <v>206</v>
       </c>
     </row>
-    <row r="11" spans="1:6" ht="52.2" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:6" ht="52.25" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A11" s="25" t="s">
         <v>207</v>
       </c>
@@ -4859,7 +4890,7 @@
         <v>212</v>
       </c>
     </row>
-    <row r="12" spans="1:6" ht="48" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:6" ht="48" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A12" s="25" t="s">
         <v>213</v>
       </c>
@@ -4887,16 +4918,16 @@
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
   <dimension ref="A1:B8"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultColWidth="8.90625" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="24.6640625" style="49" customWidth="1"/>
-    <col min="2" max="2" width="27.77734375" style="5" customWidth="1"/>
-    <col min="3" max="16384" width="8.88671875" style="5"/>
+    <col min="1" max="1" width="24.6328125" style="49" customWidth="1"/>
+    <col min="2" max="2" width="27.81640625" style="5" customWidth="1"/>
+    <col min="3" max="16384" width="8.90625" style="5"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A1" s="50" t="s">
         <v>229</v>
       </c>
@@ -4904,7 +4935,7 @@
         <v>230</v>
       </c>
     </row>
-    <row r="2" spans="1:2" ht="114" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:2" ht="114" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A2" s="50" t="s">
         <v>231</v>
       </c>
@@ -4912,7 +4943,7 @@
         <v>232</v>
       </c>
     </row>
-    <row r="3" spans="1:2" ht="72" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:2" ht="72.5" x14ac:dyDescent="0.35">
       <c r="A3" s="50" t="s">
         <v>233</v>
       </c>
@@ -4920,7 +4951,7 @@
         <v>243</v>
       </c>
     </row>
-    <row r="4" spans="1:2" ht="72" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:2" ht="72.5" x14ac:dyDescent="0.35">
       <c r="A4" s="50" t="s">
         <v>234</v>
       </c>
@@ -4928,7 +4959,7 @@
         <v>235</v>
       </c>
     </row>
-    <row r="5" spans="1:2" ht="86.4" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:2" ht="87" x14ac:dyDescent="0.35">
       <c r="A5" s="50" t="s">
         <v>236</v>
       </c>
@@ -4936,7 +4967,7 @@
         <v>244</v>
       </c>
     </row>
-    <row r="6" spans="1:2" ht="57.6" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:2" ht="58" x14ac:dyDescent="0.35">
       <c r="A6" s="50" t="s">
         <v>237</v>
       </c>
@@ -4944,7 +4975,7 @@
         <v>238</v>
       </c>
     </row>
-    <row r="7" spans="1:2" ht="72" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:2" ht="72.5" x14ac:dyDescent="0.35">
       <c r="A7" s="50" t="s">
         <v>239</v>
       </c>
@@ -4952,7 +4983,7 @@
         <v>240</v>
       </c>
     </row>
-    <row r="8" spans="1:2" ht="86.4" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:2" ht="87" x14ac:dyDescent="0.35">
       <c r="A8" s="50" t="s">
         <v>241</v>
       </c>
@@ -4966,21 +4997,21 @@
 </file>
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0400-000000000000}">
   <dimension ref="A1:K9"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="13.109375" style="22" customWidth="1"/>
-    <col min="2" max="2" width="28.33203125" style="15" customWidth="1"/>
-    <col min="3" max="3" width="24.5546875" style="15" customWidth="1"/>
-    <col min="4" max="4" width="27.44140625" customWidth="1"/>
+    <col min="1" max="1" width="13.08984375" style="22" customWidth="1"/>
+    <col min="2" max="2" width="28.36328125" style="15" customWidth="1"/>
+    <col min="3" max="3" width="24.54296875" style="15" customWidth="1"/>
+    <col min="4" max="4" width="27.453125" customWidth="1"/>
     <col min="5" max="6" width="30" customWidth="1"/>
-    <col min="7" max="7" width="21.88671875" customWidth="1"/>
-    <col min="8" max="8" width="25.77734375" style="23" customWidth="1"/>
-    <col min="9" max="9" width="21.5546875" customWidth="1"/>
+    <col min="7" max="7" width="21.90625" customWidth="1"/>
+    <col min="8" max="8" width="25.81640625" style="23" customWidth="1"/>
+    <col min="9" max="9" width="21.54296875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A1" s="35" t="s">
         <v>79</v>
       </c>
@@ -4991,7 +5022,7 @@
         <v>81</v>
       </c>
     </row>
-    <row r="2" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A2" s="35" t="s">
         <v>53</v>
       </c>
@@ -5002,7 +5033,7 @@
         <v>83</v>
       </c>
     </row>
-    <row r="3" spans="1:11" ht="57.6" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:11" ht="58" x14ac:dyDescent="0.35">
       <c r="A3" s="35" t="s">
         <v>88</v>
       </c>
@@ -5013,7 +5044,7 @@
         <v>89</v>
       </c>
     </row>
-    <row r="4" spans="1:11" ht="43.2" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:11" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A4" s="35" t="s">
         <v>84</v>
       </c>
@@ -5024,8 +5055,8 @@
         <v>86</v>
       </c>
     </row>
-    <row r="5" spans="1:11" ht="156.6" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A5" s="58" t="s">
+    <row r="5" spans="1:11" ht="156.65" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A5" s="63" t="s">
         <v>87</v>
       </c>
       <c r="B5" s="38" t="s">
@@ -5050,8 +5081,8 @@
         <v>98</v>
       </c>
     </row>
-    <row r="6" spans="1:11" ht="166.2" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A6" s="58"/>
+    <row r="6" spans="1:11" ht="166.25" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A6" s="63"/>
       <c r="B6" s="38" t="s">
         <v>245</v>
       </c>
@@ -5077,8 +5108,8 @@
       <c r="J6" s="5"/>
       <c r="K6" s="5"/>
     </row>
-    <row r="7" spans="1:11" ht="122.4" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A7" s="58"/>
+    <row r="7" spans="1:11" ht="122.4" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A7" s="63"/>
       <c r="B7" s="38" t="s">
         <v>94</v>
       </c>
@@ -5106,7 +5137,7 @@
       <c r="J7" s="5"/>
       <c r="K7" s="5"/>
     </row>
-    <row r="8" spans="1:11" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:11" ht="29" x14ac:dyDescent="0.35">
       <c r="A8" s="35" t="s">
         <v>90</v>
       </c>
@@ -5117,7 +5148,7 @@
         <v>92</v>
       </c>
     </row>
-    <row r="9" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A9" s="35" t="s">
         <v>56</v>
       </c>
@@ -5134,25 +5165,25 @@
 </file>
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0500-000000000000}">
   <dimension ref="A1:C24"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultColWidth="8.90625" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="22.88671875" style="2" customWidth="1"/>
-    <col min="2" max="2" width="31.77734375" style="24" customWidth="1"/>
-    <col min="3" max="3" width="42.77734375" style="5" customWidth="1"/>
-    <col min="4" max="16384" width="8.88671875" style="5"/>
+    <col min="1" max="1" width="22.90625" style="2" customWidth="1"/>
+    <col min="2" max="2" width="31.81640625" style="24" customWidth="1"/>
+    <col min="3" max="3" width="42.81640625" style="5" customWidth="1"/>
+    <col min="4" max="16384" width="8.90625" style="5"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" ht="40.799999999999997" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="62" t="s">
+    <row r="1" spans="1:3" ht="40.75" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A1" s="67" t="s">
         <v>152</v>
       </c>
-      <c r="B1" s="62"/>
-      <c r="C1" s="62"/>
-    </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A2" s="59" t="s">
+      <c r="B1" s="67"/>
+      <c r="C1" s="67"/>
+    </row>
+    <row r="2" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A2" s="64" t="s">
         <v>135</v>
       </c>
       <c r="B2" s="32" t="s">
@@ -5162,8 +5193,8 @@
         <v>111</v>
       </c>
     </row>
-    <row r="3" spans="1:3" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A3" s="59"/>
+    <row r="3" spans="1:3" ht="29" x14ac:dyDescent="0.35">
+      <c r="A3" s="64"/>
       <c r="B3" s="32" t="s">
         <v>108</v>
       </c>
@@ -5171,8 +5202,8 @@
         <v>148</v>
       </c>
     </row>
-    <row r="4" spans="1:3" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A4" s="59"/>
+    <row r="4" spans="1:3" ht="29" x14ac:dyDescent="0.35">
+      <c r="A4" s="64"/>
       <c r="B4" s="32" t="s">
         <v>109</v>
       </c>
@@ -5180,8 +5211,8 @@
         <v>153</v>
       </c>
     </row>
-    <row r="5" spans="1:3" ht="100.8" x14ac:dyDescent="0.3">
-      <c r="A5" s="59"/>
+    <row r="5" spans="1:3" ht="101.5" x14ac:dyDescent="0.35">
+      <c r="A5" s="64"/>
       <c r="B5" s="32" t="s">
         <v>110</v>
       </c>
@@ -5189,8 +5220,8 @@
         <v>113</v>
       </c>
     </row>
-    <row r="6" spans="1:3" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A6" s="59"/>
+    <row r="6" spans="1:3" ht="29" x14ac:dyDescent="0.35">
+      <c r="A6" s="64"/>
       <c r="B6" s="32" t="s">
         <v>138</v>
       </c>
@@ -5198,8 +5229,8 @@
         <v>139</v>
       </c>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A7" s="59"/>
+    <row r="7" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A7" s="64"/>
       <c r="B7" s="32" t="s">
         <v>147</v>
       </c>
@@ -5207,8 +5238,8 @@
         <v>154</v>
       </c>
     </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A8" s="59"/>
+    <row r="8" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A8" s="64"/>
       <c r="B8" s="32" t="s">
         <v>112</v>
       </c>
@@ -5216,8 +5247,8 @@
         <v>145</v>
       </c>
     </row>
-    <row r="9" spans="1:3" ht="57.6" x14ac:dyDescent="0.3">
-      <c r="A9" s="61" t="s">
+    <row r="9" spans="1:3" ht="58" x14ac:dyDescent="0.35">
+      <c r="A9" s="66" t="s">
         <v>136</v>
       </c>
       <c r="B9" s="27" t="s">
@@ -5227,8 +5258,8 @@
         <v>146</v>
       </c>
     </row>
-    <row r="10" spans="1:3" ht="43.2" x14ac:dyDescent="0.3">
-      <c r="A10" s="61"/>
+    <row r="10" spans="1:3" ht="43.5" x14ac:dyDescent="0.35">
+      <c r="A10" s="66"/>
       <c r="B10" s="27" t="s">
         <v>114</v>
       </c>
@@ -5236,8 +5267,8 @@
         <v>115</v>
       </c>
     </row>
-    <row r="11" spans="1:3" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A11" s="61"/>
+    <row r="11" spans="1:3" ht="29" x14ac:dyDescent="0.35">
+      <c r="A11" s="66"/>
       <c r="B11" s="27" t="s">
         <v>141</v>
       </c>
@@ -5245,8 +5276,8 @@
         <v>142</v>
       </c>
     </row>
-    <row r="12" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A12" s="61"/>
+    <row r="12" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A12" s="66"/>
       <c r="B12" s="28" t="s">
         <v>116</v>
       </c>
@@ -5254,8 +5285,8 @@
         <v>117</v>
       </c>
     </row>
-    <row r="13" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A13" s="61"/>
+    <row r="13" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A13" s="66"/>
       <c r="B13" s="27" t="s">
         <v>149</v>
       </c>
@@ -5263,8 +5294,8 @@
         <v>150</v>
       </c>
     </row>
-    <row r="14" spans="1:3" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A14" s="61"/>
+    <row r="14" spans="1:3" ht="29" x14ac:dyDescent="0.35">
+      <c r="A14" s="66"/>
       <c r="B14" s="28" t="s">
         <v>122</v>
       </c>
@@ -5272,15 +5303,15 @@
         <v>151</v>
       </c>
     </row>
-    <row r="15" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A15" s="61"/>
+    <row r="15" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A15" s="66"/>
       <c r="B15" s="28" t="s">
         <v>123</v>
       </c>
       <c r="C15" s="29"/>
     </row>
-    <row r="16" spans="1:3" ht="43.2" x14ac:dyDescent="0.3">
-      <c r="A16" s="61"/>
+    <row r="16" spans="1:3" ht="43.5" x14ac:dyDescent="0.35">
+      <c r="A16" s="66"/>
       <c r="B16" s="28" t="s">
         <v>118</v>
       </c>
@@ -5288,8 +5319,8 @@
         <v>119</v>
       </c>
     </row>
-    <row r="17" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A17" s="61"/>
+    <row r="17" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A17" s="66"/>
       <c r="B17" s="28" t="s">
         <v>120</v>
       </c>
@@ -5297,8 +5328,8 @@
         <v>121</v>
       </c>
     </row>
-    <row r="18" spans="1:3" ht="43.2" x14ac:dyDescent="0.3">
-      <c r="A18" s="60" t="s">
+    <row r="18" spans="1:3" ht="43.5" x14ac:dyDescent="0.35">
+      <c r="A18" s="65" t="s">
         <v>137</v>
       </c>
       <c r="B18" s="30" t="s">
@@ -5308,8 +5339,8 @@
         <v>124</v>
       </c>
     </row>
-    <row r="19" spans="1:3" ht="43.2" x14ac:dyDescent="0.3">
-      <c r="A19" s="60"/>
+    <row r="19" spans="1:3" ht="43.5" x14ac:dyDescent="0.35">
+      <c r="A19" s="65"/>
       <c r="B19" s="30" t="s">
         <v>143</v>
       </c>
@@ -5317,8 +5348,8 @@
         <v>144</v>
       </c>
     </row>
-    <row r="20" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A20" s="60"/>
+    <row r="20" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A20" s="65"/>
       <c r="B20" s="30" t="s">
         <v>125</v>
       </c>
@@ -5326,8 +5357,8 @@
         <v>126</v>
       </c>
     </row>
-    <row r="21" spans="1:3" ht="57.6" x14ac:dyDescent="0.3">
-      <c r="A21" s="60"/>
+    <row r="21" spans="1:3" ht="58" x14ac:dyDescent="0.35">
+      <c r="A21" s="65"/>
       <c r="B21" s="30" t="s">
         <v>127</v>
       </c>
@@ -5335,8 +5366,8 @@
         <v>128</v>
       </c>
     </row>
-    <row r="22" spans="1:3" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A22" s="60"/>
+    <row r="22" spans="1:3" ht="29" x14ac:dyDescent="0.35">
+      <c r="A22" s="65"/>
       <c r="B22" s="30" t="s">
         <v>129</v>
       </c>
@@ -5344,8 +5375,8 @@
         <v>130</v>
       </c>
     </row>
-    <row r="23" spans="1:3" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A23" s="60"/>
+    <row r="23" spans="1:3" ht="29" x14ac:dyDescent="0.35">
+      <c r="A23" s="65"/>
       <c r="B23" s="30" t="s">
         <v>131</v>
       </c>
@@ -5353,8 +5384,8 @@
         <v>132</v>
       </c>
     </row>
-    <row r="24" spans="1:3" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A24" s="60"/>
+    <row r="24" spans="1:3" ht="29" x14ac:dyDescent="0.35">
+      <c r="A24" s="65"/>
       <c r="B24" s="30" t="s">
         <v>133</v>
       </c>
@@ -5375,17 +5406,17 @@
 </file>
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0600-000000000000}">
   <dimension ref="A1:F8"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="19.77734375" style="14" customWidth="1"/>
+    <col min="1" max="1" width="19.81640625" style="14" customWidth="1"/>
     <col min="2" max="2" width="35" style="16" customWidth="1"/>
-    <col min="3" max="3" width="25.88671875" style="16" customWidth="1"/>
-    <col min="4" max="4" width="17.88671875" style="1" customWidth="1"/>
+    <col min="3" max="3" width="25.90625" style="16" customWidth="1"/>
+    <col min="4" max="4" width="17.90625" style="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" s="17" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:6" s="17" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A1" s="8" t="s">
         <v>47</v>
       </c>
@@ -5401,7 +5432,7 @@
       <c r="E1" s="13"/>
       <c r="F1" s="13"/>
     </row>
-    <row r="2" spans="1:6" ht="49.8" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:6" ht="49.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A2" s="8" t="s">
         <v>48</v>
       </c>
@@ -5417,7 +5448,7 @@
       <c r="E2" s="5"/>
       <c r="F2" s="5"/>
     </row>
-    <row r="3" spans="1:6" ht="42" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:6" ht="42" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A3" s="8" t="s">
         <v>49</v>
       </c>
@@ -5433,7 +5464,7 @@
       <c r="E3" s="5"/>
       <c r="F3" s="5"/>
     </row>
-    <row r="4" spans="1:6" ht="79.2" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:6" ht="86.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A4" s="8" t="s">
         <v>50</v>
       </c>
@@ -5449,7 +5480,7 @@
       <c r="E4" s="5"/>
       <c r="F4" s="5"/>
     </row>
-    <row r="5" spans="1:6" ht="77.400000000000006" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:6" ht="77.400000000000006" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A5" s="8" t="s">
         <v>51</v>
       </c>
@@ -5465,7 +5496,7 @@
       <c r="E5" s="5"/>
       <c r="F5" s="5"/>
     </row>
-    <row r="6" spans="1:6" ht="54.6" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:6" ht="54.65" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A6" s="8" t="s">
         <v>52</v>
       </c>
@@ -5481,7 +5512,7 @@
       <c r="E6" s="5"/>
       <c r="F6" s="5"/>
     </row>
-    <row r="7" spans="1:6" ht="66" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:6" ht="66" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A7" s="8" t="s">
         <v>53</v>
       </c>
@@ -5497,7 +5528,7 @@
       <c r="E7" s="5"/>
       <c r="F7" s="5"/>
     </row>
-    <row r="8" spans="1:6" ht="50.4" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:6" ht="50.4" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A8" s="8" t="s">
         <v>54</v>
       </c>
@@ -5519,23 +5550,23 @@
 </file>
 
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0700-000000000000}">
   <dimension ref="A1:C21"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="23.88671875" style="24" customWidth="1"/>
-    <col min="2" max="2" width="34.5546875" style="53" customWidth="1"/>
-    <col min="3" max="3" width="17.44140625" style="53" customWidth="1"/>
+    <col min="1" max="1" width="23.90625" style="24" customWidth="1"/>
+    <col min="2" max="2" width="34.54296875" style="53" customWidth="1"/>
+    <col min="3" max="3" width="17.453125" style="53" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" ht="18" x14ac:dyDescent="0.35">
-      <c r="A1" s="63" t="s">
+    <row r="1" spans="1:3" ht="18.5" x14ac:dyDescent="0.45">
+      <c r="A1" s="68" t="s">
         <v>246</v>
       </c>
-      <c r="B1" s="63"/>
-      <c r="C1" s="63"/>
-    </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="B1" s="68"/>
+      <c r="C1" s="68"/>
+    </row>
+    <row r="2" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A2" s="2"/>
       <c r="B2" s="2" t="s">
         <v>263</v>
@@ -5544,7 +5575,7 @@
         <v>56</v>
       </c>
     </row>
-    <row r="3" spans="1:3" ht="55.8" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:3" ht="55.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A3" s="52" t="s">
         <v>48</v>
       </c>
@@ -5555,7 +5586,7 @@
         <v>265</v>
       </c>
     </row>
-    <row r="4" spans="1:3" ht="52.8" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:3" ht="52.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A4" s="52" t="s">
         <v>247</v>
       </c>
@@ -5566,7 +5597,7 @@
         <v>266</v>
       </c>
     </row>
-    <row r="5" spans="1:3" ht="75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:3" ht="75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A5" s="52" t="s">
         <v>248</v>
       </c>
@@ -5577,7 +5608,7 @@
         <v>268</v>
       </c>
     </row>
-    <row r="6" spans="1:3" ht="55.2" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:3" ht="55.25" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A6" s="52" t="s">
         <v>249</v>
       </c>
@@ -5588,7 +5619,7 @@
         <v>271</v>
       </c>
     </row>
-    <row r="7" spans="1:3" ht="52.8" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:3" ht="52.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A7" s="52" t="s">
         <v>250</v>
       </c>
@@ -5599,14 +5630,14 @@
         <v>273</v>
       </c>
     </row>
-    <row r="9" spans="1:3" ht="18" x14ac:dyDescent="0.35">
-      <c r="A9" s="63" t="s">
+    <row r="9" spans="1:3" ht="18.5" x14ac:dyDescent="0.45">
+      <c r="A9" s="68" t="s">
         <v>251</v>
       </c>
-      <c r="B9" s="63"/>
-      <c r="C9" s="63"/>
-    </row>
-    <row r="10" spans="1:3" ht="51" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B9" s="68"/>
+      <c r="C9" s="68"/>
+    </row>
+    <row r="10" spans="1:3" ht="51" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A10" s="52" t="s">
         <v>252</v>
       </c>
@@ -5614,7 +5645,7 @@
         <v>274</v>
       </c>
     </row>
-    <row r="11" spans="1:3" ht="58.2" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:3" ht="58.25" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A11" s="52" t="s">
         <v>253</v>
       </c>
@@ -5622,7 +5653,7 @@
         <v>275</v>
       </c>
     </row>
-    <row r="12" spans="1:3" ht="63" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:3" ht="63" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A12" s="52" t="s">
         <v>254</v>
       </c>
@@ -5630,7 +5661,7 @@
         <v>276</v>
       </c>
     </row>
-    <row r="13" spans="1:3" ht="54" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:3" ht="54" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A13" s="52" t="s">
         <v>255</v>
       </c>
@@ -5638,7 +5669,7 @@
         <v>277</v>
       </c>
     </row>
-    <row r="14" spans="1:3" ht="73.2" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:3" ht="73.25" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A14" s="52" t="s">
         <v>257</v>
       </c>
@@ -5646,7 +5677,7 @@
         <v>278</v>
       </c>
     </row>
-    <row r="15" spans="1:3" ht="55.2" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:3" ht="55.25" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A15" s="52" t="s">
         <v>256</v>
       </c>
@@ -5654,14 +5685,14 @@
         <v>279</v>
       </c>
     </row>
-    <row r="17" spans="1:3" ht="18" x14ac:dyDescent="0.35">
-      <c r="A17" s="63" t="s">
+    <row r="17" spans="1:3" ht="18.5" x14ac:dyDescent="0.45">
+      <c r="A17" s="68" t="s">
         <v>258</v>
       </c>
-      <c r="B17" s="63"/>
-      <c r="C17" s="63"/>
-    </row>
-    <row r="18" spans="1:3" ht="58.2" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B17" s="68"/>
+      <c r="C17" s="68"/>
+    </row>
+    <row r="18" spans="1:3" ht="58.25" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A18" s="52" t="s">
         <v>259</v>
       </c>
@@ -5672,7 +5703,7 @@
         <v>280</v>
       </c>
     </row>
-    <row r="19" spans="1:3" ht="73.8" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:3" ht="73.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A19" s="52" t="s">
         <v>260</v>
       </c>
@@ -5683,7 +5714,7 @@
         <v>280</v>
       </c>
     </row>
-    <row r="20" spans="1:3" ht="57.6" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:3" ht="57.65" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A20" s="52" t="s">
         <v>261</v>
       </c>
@@ -5694,7 +5725,7 @@
         <v>285</v>
       </c>
     </row>
-    <row r="21" spans="1:3" ht="57.6" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:3" ht="57.65" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A21" s="52" t="s">
         <v>262</v>
       </c>

</xml_diff>